<commit_message>
Despliegue en AWS y documentos actualizados
</commit_message>
<xml_diff>
--- a/Primer Entregable/QA02-Casos de Pruebas - TechStore.xlsx
+++ b/Primer Entregable/QA02-Casos de Pruebas - TechStore.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebasrc\Downloads\ecommerce-tech\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{993C91C8-6559-4CB6-9010-C3F237B9433B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFD5414E-1B87-48E7-8E5E-6EAB4ED7744D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
     <t>Plataforma:</t>
   </si>
   <si>
-    <t>Web – TechStore v1.0 – Ambiente QA en Azure App Service (&lt;URL_QA&gt;) – Chrome, Edge, Firefox</t>
+    <t>Web – TechStore v1.0 – Ambiente QA en AWS Elastic Beanstalk (&lt;URL_QA&gt;) – Chrome, Edge, Firefox</t>
   </si>
   <si>
     <t>Módulo (Suite)</t>
@@ -2058,7 +2058,7 @@
     <t>Verificar tiempo de respuesta del catálogo</t>
   </si>
   <si>
-    <t>Herramienta: Grafana k6 / JMeter – Ambiente QA (Azure).</t>
+    <t>Herramienta: Grafana k6 / JMeter – Ambiente QA (AWS).</t>
   </si>
   <si>
     <t>1. Prueba de carga a GET /api/products con 20 usuarios virtuales concurrentes durante 5 minutos.</t>
@@ -2076,7 +2076,7 @@
     <t>Verificar tiempo de cálculo del carrito (motor de precios)</t>
   </si>
   <si>
-    <t>Herramienta: Grafana k6 – Ambiente QA (Azure).</t>
+    <t>Herramienta: Grafana k6 – Ambiente QA (AWS).</t>
   </si>
   <si>
     <t>1. Carga a POST /api/cart/items con 10 usuarios autenticados durante 3 minutos.</t>
@@ -2184,13 +2184,13 @@
     <t>Verificar comunicación cifrada</t>
   </si>
   <si>
-    <t>Herramienta: Playwright (API) – Producción (Azure).</t>
+    <t>Herramienta: Playwright (API) – Producción (AWS).</t>
   </si>
   <si>
     <t>1. Acceder al sitio de producción por http:// y revisar el certificado.</t>
   </si>
   <si>
-    <t>Redirección automática a https:// (App Service con 'Solo HTTPS').</t>
+    <t>Redirección automática a https:// (CloudFront con 'Redirect HTTP to HTTPS').</t>
   </si>
   <si>
     <t>RNF-08 (ver QA01 sección 2.4). Script: tests/e2e/specs/12-no-funcionales.spec.ts</t>
@@ -2220,7 +2220,7 @@
     <t>Verificar manejo seguro de errores</t>
   </si>
   <si>
-    <t>1. Provocar un error (ID mal formado, cuerpo JSON inválido) en endpoints de la API en el ambiente de Azure.</t>
+    <t>1. Provocar un error (ID mal formado, cuerpo JSON inválido) en endpoints de la API en el ambiente de AWS.</t>
   </si>
   <si>
     <t>Respuesta 4xx controlada; no se expone stack trace, rutas del servidor ni cadena de conexión.</t>
@@ -2313,7 +2313,7 @@
     <t>Verificar disponibilidad del servicio</t>
   </si>
   <si>
-    <t>Herramienta: Playwright + Azure Application Insights.</t>
+    <t>Herramienta: Playwright + Amazon CloudWatch Synthetics.</t>
   </si>
   <si>
     <t>1. Sondeo automático de la web y la API (10 solicitudes) y monitoreo continuo cada 5 minutos en producción.</t>
@@ -2331,13 +2331,13 @@
     <t>Verificar respaldo y recuperación de la base de datos</t>
   </si>
   <si>
-    <t>Herramienta: Azure CLI (test-restore.ps1).</t>
-  </si>
-  <si>
-    <t>1. Script que restaura la base a un punto en el tiempo (PITR) en una base nueva, verifica su estado y la elimina.</t>
-  </si>
-  <si>
-    <t>Base restaurada Online en &lt; 30 min.</t>
+    <t>Herramienta: AWS CLI (scripts/aws/test-restore.ps1).</t>
+  </si>
+  <si>
+    <t>1. Script que restaura la instancia RDS a un punto en el tiempo en una instancia nueva, verifica que quede disponible y la elimina.</t>
+  </si>
+  <si>
+    <t>Instancia restaurada disponible en &lt; 60 min.</t>
   </si>
   <si>
     <t>RNF-16 (ver QA01 sección 2.4). Script: tests/e2e/specs/12-no-funcionales.spec.ts</t>
@@ -2373,10 +2373,10 @@
     <t>Verificar instalabilidad del sistema</t>
   </si>
   <si>
-    <t>Herramienta: Azure CLI (deploy.ps1) + Playwright.</t>
-  </si>
-  <si>
-    <t>1. Script de despliegue (compilación, publicación y subida al App Service) seguido de la prueba de humo @smoke.</t>
+    <t>Herramienta: AWS CLI (scripts/aws/deploy.ps1) + Playwright.</t>
+  </si>
+  <si>
+    <t>1. Script de despliegue (compilación, publicación y nueva versión en Elastic Beanstalk) seguido de la prueba de humo @smoke.</t>
   </si>
   <si>
     <t>Sistema operativo en &lt; 60 min y prueba de humo aprobada.</t>
@@ -39239,8 +39239,8 @@
   <autoFilter ref="B7:L147" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="4">
     <mergeCell ref="C4:G4"/>
+    <mergeCell ref="C5:G5"/>
     <mergeCell ref="C2:G2"/>
-    <mergeCell ref="C5:G5"/>
     <mergeCell ref="C3:G3"/>
   </mergeCells>
   <conditionalFormatting sqref="K8:K147">
@@ -39289,12 +39289,12 @@
     <col min="7" max="7" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="13" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="14" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:7" ht="14" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
         <v>730</v>
       </c>
@@ -39314,7 +39314,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="5" spans="2:7" ht="25" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="14" t="s">
         <v>735</v>
       </c>
@@ -39404,7 +39404,7 @@
       </c>
       <c r="G9" s="15"/>
     </row>
-    <row r="10" spans="2:7" ht="25" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="14" t="s">
         <v>750</v>
       </c>
@@ -39496,7 +39496,7 @@
       </c>
       <c r="G14" s="15"/>
     </row>
-    <row r="15" spans="2:7" ht="25" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="14" t="s">
         <v>766</v>
       </c>
@@ -39550,7 +39550,7 @@
       </c>
       <c r="G17" s="15"/>
     </row>
-    <row r="18" spans="2:7" ht="25" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="14" t="s">
         <v>775</v>
       </c>
@@ -39604,7 +39604,7 @@
       </c>
       <c r="G20" s="15"/>
     </row>
-    <row r="21" spans="2:7" ht="25" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="14" t="s">
         <v>784</v>
       </c>
@@ -39658,7 +39658,7 @@
       </c>
       <c r="G23" s="15"/>
     </row>
-    <row r="24" spans="2:7" ht="25" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="14" t="s">
         <v>793</v>
       </c>
@@ -39732,7 +39732,7 @@
         <v>804</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="25" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="14" t="s">
         <v>805</v>
       </c>
@@ -40093,12 +40093,12 @@
     <col min="3" max="3" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="13" t="s">
         <v>845</v>
       </c>
     </row>
-    <row r="4" spans="2:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="16" t="s">
         <v>846</v>
       </c>
@@ -40107,7 +40107,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="16" t="s">
         <v>847</v>
       </c>
@@ -40116,7 +40116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="16" t="s">
         <v>848</v>
       </c>
@@ -40125,7 +40125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="16" t="s">
         <v>849</v>
       </c>
@@ -40134,7 +40134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="16" t="s">
         <v>27</v>
       </c>
@@ -40143,7 +40143,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="9" spans="2:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="16" t="s">
         <v>850</v>
       </c>
@@ -40152,7 +40152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="16" t="s">
         <v>851</v>
       </c>
@@ -40160,7 +40160,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="16" t="s">
         <v>852</v>
       </c>
@@ -40168,7 +40168,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="2:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="16" t="s">
         <v>853</v>
       </c>

</xml_diff>